<commit_message>
bugs are fixed except mandir
</commit_message>
<xml_diff>
--- a/task_list.xlsx
+++ b/task_list.xlsx
@@ -14,7 +14,7 @@
   </HeadingPairs>
   <TitlesOfParts>
     <vt:vector size="1" baseType="lpstr">
-      <vt:lpstr>Last 15 Days Work</vt:lpstr>
+      <vt:lpstr>Task List</vt:lpstr>
     </vt:vector>
   </TitlesOfParts>
 </Properties>
@@ -415,14 +415,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Last 15 Days Work" sheetId="1" r:id="rId1"/>
+    <sheet name="Task List" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1261,9 +1261,32 @@
         <v>iOS update completed. Podfile, Runner.xcodeproj/project.pbxproj, Info.plist, GeneratedPluginRegistrant.m updated.</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>AstroBharatai</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Open Kundli Feature</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Development</v>
+      </c>
+      <c r="E37" t="str">
+        <v>15-03-2026</v>
+      </c>
+      <c r="F37" t="str">
+        <v>15-03-2026</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Open kundli feature is done.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>